<commit_message>
Made changes on RMMM_CryptoBroker.xlsx and the arc42 documentation.
</commit_message>
<xml_diff>
--- a/docs/RMMM_CryptoBroker.xlsx
+++ b/docs/RMMM_CryptoBroker.xlsx
@@ -127,7 +127,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -149,11 +149,55 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -194,6 +238,8 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -559,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -666,6 +712,17 @@
           <t>Technische Risiken</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="14" t="n"/>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="14" t="n"/>
+      <c r="H4" s="14" t="n"/>
+      <c r="I4" s="14" t="n"/>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="14" t="n"/>
+      <c r="L4" s="15" t="n"/>
     </row>
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -737,32 +794,32 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Fiktive Währung: fehlerhafte Kursgenerierung
-Im aktuellen Sprint wurde eine fiktive Kryptowährung eingeführt, deren Kursverlauf algorithmisch generiert wird statt von einer externen API zu kommen. Fehler in der Generierungslogik (z. B. negative Kurse, Integer-Overflows, fehlende History-Tabelle) können zu falschen Portfolio-Berechnungen oder Abstürzen führen.</t>
+          <t>SQLite Race Conditions bei gleichzeitigen Trades
+SQLite erlaubt nur einen Schreibzugriff gleichzeitig. Bei mehreren parallelen BUY/SELL-Requests (z. B. mehrere Browser-Tabs) können Transaktionen verloren gehen oder der Kontostand inkonsistent werden.</t>
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="9" t="n">
-        <v>20</v>
+      <c r="F6" s="8" t="n">
+        <v>10</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Unit-Tests für den Kurs-Generator schreiben (Randwerte: Preis &gt; 0, keine NaN/Inf-Werte). Validierung im CoinSyncService: vor INSERT prüfen, ob generierter Preis &gt; 0 und endlich. Separate History-Tabelle für fiktive Währung analog zu realen Coins anlegen.</t>
+          <t>Write-Ahead Logging (WAL) für SQLite aktivieren. Datenbankzugriffe in MarketService durch einen Lock (threading.Lock) serialisieren. Langfristig: Migration zu PostgreSQL für ACID-konforme Parallelzugriffe.</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Portfolio-Gesamtwert springt unrealistisch; Fehler beim Öffnen der Coin-Detailseite der fiktiven Währung; Transaktionen mit negativem Wert in der DB.</t>
+          <t>"database is locked"-Fehler in den Logs; Portfolio-Saldo weicht von Summe der Transaktionen ab.</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Fiktive Währung aus dem Dashboard ausblenden, bis Kurs-Generator validiert ist. Datenbankeinträge mit ungültigen Preisen löschen und Tabelle neu befüllen. Hotfix-Branch direkt auf main mergen.</t>
+          <t>Anwendung neu starten (löst Lock-Situation). Inkonsistente Transaktionen in der DB manuell identifizieren und korrigieren. Bei Wiederholung: SQLite durch PostgreSQL ersetzen.</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
@@ -772,7 +829,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -782,130 +839,141 @@
       </c>
     </row>
     <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>T-03</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Technisch</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>SQLite Race Conditions bei gleichzeitigen Trades
-SQLite erlaubt nur einen Schreibzugriff gleichzeitig. Bei mehreren parallelen BUY/SELL-Requests (z. B. mehrere Browser-Tabs) können Transaktionen verloren gehen oder der Kontostand inkonsistent werden.</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Write-Ahead Logging (WAL) für SQLite aktivieren. Datenbankzugriffe in MarketService durch einen Lock (threading.Lock) serialisieren. Langfristig: Migration zu PostgreSQL für ACID-konforme Parallelzugriffe.</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>"database is locked"-Fehler in den Logs; Portfolio-Saldo weicht von Summe der Transaktionen ab.</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>Anwendung neu starten (löst Lock-Situation). Inkonsistente Transaktionen in der DB manuell identifizieren und korrigieren. Bei Wiederholung: SQLite durch PostgreSQL ersetzen.</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>Sara</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>21.04.2026</t>
-        </is>
-      </c>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Projektrisiken</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n"/>
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="14" t="n"/>
+      <c r="E7" s="14" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="14" t="n"/>
+      <c r="H7" s="14" t="n"/>
+      <c r="I7" s="14" t="n"/>
+      <c r="J7" s="14" t="n"/>
+      <c r="K7" s="14" t="n"/>
+      <c r="L7" s="15" t="n"/>
     </row>
     <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>T-04</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Technisch</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Unsicherer Secret Key für Flask-Sessions
-Der Session-Secret-Key ist als Klartext "change-me-in-production" im Quellcode hinterlegt (app.py). Ein Angreifer mit Zugang zum Repository kann Sessions fälschen und sich als beliebiger Nutzer einloggen.</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Teamausfall (Krankheit / Prüfungsphase)
+Das Team besteht aus nur 4 Personen. Fällt ein Mitglied längerfristig aus (Krankheit, Prüfungsstress), können Sprint-Ziele nicht gehalten werden. Besonders kritisch, wenn Wissen über einen Teilbereich nur bei einer Person liegt.</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Secret Key aus Quellcode entfernen und in .env-Datei auslagern (bereits als .env vorgesehen). python-dotenv verwenden, um den Key beim Start zu laden. .env in .gitignore aufnehmen und aus Git-History entfernen (git filter-branch oder BFG).</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>Secret Key im öffentlichen Repository sichtbar; Session-Cookie kann außerhalb der App generiert werden.</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>Sofortiger Commit mit zufälligem, generiertem Key (z. B. secrets.token_hex(32)). Alle aktiven Sessions durch Änderung des Keys invalidieren. Zugriffsrechte für das Repository prüfen.</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="E8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Wissenstransfer durch regelmäßige Pair-Programming-Sessions und Code-Reviews. Kritische Komponenten (z. B. CoinSyncService) dokumentieren. Aufgaben nicht dauerhaft einer einzigen Person zuordnen.</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>Mehrere Sprints ohne Pull-Request einer Person; Standup-Meetings zeigen blockierten Fortschritt.</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>Aufgaben des ausgefallenen Mitglieds im Team neu verteilen. Sprint-Scope reduzieren und Dozenten frühzeitig informieren.</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>Julian</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="L8" s="11" t="inlineStr">
         <is>
           <t>21.04.2026</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Projektrisiken</t>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Projekt</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Scope Creep: unkontrolliertes Feature-Wachstum
+Neue Ideen (z. B. weitere fiktive Währungen, Echtzeit-WebSockets, Charts) werden ad-hoc zum Sprint hinzugefügt, ohne das bestehende Backlog anzupassen. Bestehende Features werden dadurch nicht fertiggestellt oder ausreichend getestet.</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Strikte Definition-of-Done pro Sprint einhalten. Neue Features zunächst ins Backlog aufnehmen und erst in folgenden Sprints planen. Sprint-Ziel zu Beginn schriftlich fixieren.</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>Sprint-Ziele werden nicht abgeschlossen; Anzahl offener Issues wächst schneller als Issues geschlossen werden.</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>Sprint-Scope einfrieren; angefangene, aber nicht fertige Features in separaten Feature-Branches parken und erst nach Abschluss des Kern-Sprints mergen.</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Lucas</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>21.04.2026</t>
         </is>
       </c>
     </row>
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>P-03</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -915,32 +983,32 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Teamausfall (Krankheit / Prüfungsphase)
-Das Team besteht aus nur 4 Personen. Fällt ein Mitglied längerfristig aus (Krankheit, Prüfungsstress), können Sprint-Ziele nicht gehalten werden. Besonders kritisch, wenn Wissen über einen Teilbereich nur bei einer Person liegt.</t>
+          <t>Fehlende automatisierte Tests
+Unit-Test-Coverage ist laut arc42 bislang nur "geplant" (Ziel: &gt;70%). Manuelle Tests können Regressionen bei neuen Features wie der fiktiven Währung nicht zuverlässig verhindern. Fehler werden erst spät (oder in der Abgabe) entdeckt.</t>
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>3</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Wissenstransfer durch regelmäßige Pair-Programming-Sessions und Code-Reviews. Kritische Komponenten (z. B. CoinSyncService) dokumentieren. Aufgaben nicht dauerhaft einer einzigen Person zuordnen.</t>
+          <t>pytest-Framework einrichten und erste Unit-Tests für Services schreiben. CI-Pipeline (z. B. GitHub Actions) einrichten, die Tests bei jedem Push ausführt. Priorität: Tests für Portfolio-Berechnung und Trade-Ausführung.</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>Mehrere Sprints ohne Pull-Request einer Person; Standup-Meetings zeigen blockierten Fortschritt.</t>
+          <t>Regressionen nach Merges; manuelle Testläufe schlagen fehl; Kommentare im Code wie "TODO: test this".</t>
         </is>
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>Aufgaben des ausgefallenen Mitglieds im Team neu verteilen. Sprint-Scope reduzieren und Dozenten frühzeitig informieren.</t>
+          <t>Kritische Pfade (Portfolio, Trade) manuell vor jedem Release durchklicken. Defekte Features sofort im Backlog priorisieren.</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr">
@@ -950,7 +1018,7 @@
       </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
-          <t>Julian</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
@@ -962,7 +1030,7 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>P-02</t>
+          <t>P-04</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -971,172 +1039,59 @@
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>Scope Creep: unkontrolliertes Feature-Wachstum
-Neue Ideen (z. B. weitere fiktive Währungen, Echtzeit-WebSockets, Charts) werden ad-hoc zum Sprint hinzugefügt, ohne das bestehende Backlog anzupassen. Bestehende Features werden dadurch nicht fertiggestellt oder ausreichend getestet.</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>Strikte Definition-of-Done pro Sprint einhalten. Neue Features zunächst ins Backlog aufnehmen und erst in folgenden Sprints planen. Sprint-Ziel zu Beginn schriftlich fixieren.</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>Sprint-Ziele werden nicht abgeschlossen; Anzahl offener Issues wächst schneller als Issues geschlossen werden.</t>
-        </is>
-      </c>
-      <c r="I11" s="12" t="inlineStr">
-        <is>
-          <t>Sprint-Scope einfrieren; angefangene, aber nicht fertige Features in separaten Feature-Branches parken und erst nach Abschluss des Kern-Sprints mergen.</t>
-        </is>
-      </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>Lucas</t>
-        </is>
-      </c>
-      <c r="L11" s="11" t="inlineStr">
-        <is>
-          <t>21.04.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>P-03</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Projekt</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Fehlende automatisierte Tests
-Unit-Test-Coverage ist laut arc42 bislang nur "geplant" (Ziel: &gt;70%). Manuelle Tests können Regressionen bei neuen Features wie der fiktiven Währung nicht zuverlässig verhindern. Fehler werden erst spät (oder in der Abgabe) entdeckt.</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="F12" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>pytest-Framework einrichten und erste Unit-Tests für Services schreiben. CI-Pipeline (z. B. GitHub Actions) einrichten, die Tests bei jedem Push ausführt. Priorität: Tests für Portfolio-Berechnung und Trade-Ausführung.</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr">
-        <is>
-          <t>Regressionen nach Merges; manuelle Testläufe schlagen fehl; Kommentare im Code wie "TODO: test this".</t>
-        </is>
-      </c>
-      <c r="I12" s="12" t="inlineStr">
-        <is>
-          <t>Kritische Pfade (Portfolio, Trade) manuell vor jedem Release durchklicken. Defekte Features sofort im Backlog priorisieren.</t>
-        </is>
-      </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
-          <t>Sara</t>
-        </is>
-      </c>
-      <c r="L12" s="11" t="inlineStr">
-        <is>
-          <t>21.04.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>P-04</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>Projekt</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Zeitdruck vor Abgabe / Blog-Deadline
 Deadlines (Blog bis 21.04.2026 20:00 Uhr, Kommentare bis 22.04.2026) kommen regelmäßig kurzfristig. Werden Features zu spät fertiggestellt, fehlt Zeit für Dokumentation und die Abgabe ist unvollständig.</t>
         </is>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D11" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E11" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F11" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>Wöchentliche Sprints mit klaren Meilensteinen. Blog-Einträge parallel zur Entwicklung verfassen ("Living Document"). arc42 und RMMM-Liste kontinuierlich pflegen statt kurz vor Abgabe.</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>Unfertige Pull Requests kurz vor Deadline; fehlende Kapitel im arc42-Dokument.</t>
         </is>
       </c>
-      <c r="I13" s="12" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>Scope für betroffenen Sprint reduzieren, vorhandene Ergebnisse dokumentieren und abgeben (lieber vollständige Dokumentation als halbfertiger Code).</t>
         </is>
       </c>
-      <c r="J13" s="11" t="inlineStr">
+      <c r="J11" s="11" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="K13" s="11" t="inlineStr">
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>Jonathan</t>
         </is>
       </c>
-      <c r="L13" s="11" t="inlineStr">
+      <c r="L11" s="11" t="inlineStr">
         <is>
           <t>21.04.2026</t>
         </is>
       </c>
     </row>
+    <row r="12" ht="90" customHeight="1"/>
+    <row r="13" ht="90" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A3:L13"/>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A4:L4"/>
-    <mergeCell ref="A9:L9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update RMMM & arc42
</commit_message>
<xml_diff>
--- a/docs/RMMM_CryptoBroker.xlsx
+++ b/docs/RMMM_CryptoBroker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RMMM-Liste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RMMM-Liste" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RMMM-Liste'!$A$3:$L$13</definedName>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,8 +78,18 @@
       <color rgb="00276221"/>
       <sz val="10"/>
     </font>
+    <font>
+      <color rgb="009C5700"/>
+    </font>
+    <font>
+      <color rgb="00276221"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +134,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -197,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -240,6 +268,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -738,7 +775,7 @@
       <c r="C5" s="7" t="inlineStr">
         <is>
           <t>CoinGecko API-Ausfall / Rate-Limit
-Die Anwendung ruft beim Start und bei jedem Coin-Aufruf die CoinGecko REST API ab (Free Tier: 240 req/min). Bei API-Ausfall oder Überschreitung des Limits stehen keine aktuellen Marktdaten zur Verfügung, das Dashboard zeigt veraltete oder keine Preise.</t>
+Die Anwendung ruft beim Start und bei jedem Coin-Aufruf die CoinGecko REST API ab (Demo API Key: ~30 req/min). Bei API-Ausfall oder Überschreitung des Limits stehen keine aktuellen Marktdaten zur Verfügung, das Dashboard zeigt veraltete oder keine Preise.</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
@@ -752,7 +789,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Lokales Caching der zuletzt abgerufenen Coin-Daten in der SQLite-DB implementieren. Exponential-Backoff und Retry-Logik im CoinSyncService einbauen. API-Key auf bezahlten Tier upgraden, falls nötig.</t>
+          <t>Lokales Caching der letzten Coin-Daten in SQLite implementiert. CoinSyncService fängt API-Fehler ab und fällt auf gecachte Daten zurück. Risiko bleibt strukturell bestehen (externe Abhängigkeit), ist aber durch Caching mitigiert.</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -765,9 +802,10 @@
           <t>Dashboard auf gecachte DB-Daten zurückfallen lassen mit sichtbarem Hinweis "Daten könnten veraltet sein (Stand: HH:MM)". Manuelles Retry nach 60 Sekunden.</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>Mitigiert
+(externe API-Abhängigkeit bleibt bestehen)</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -777,7 +815,7 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>27.06.2026</t>
         </is>
       </c>
     </row>
@@ -809,7 +847,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Write-Ahead Logging (WAL) für SQLite aktivieren. Datenbankzugriffe in MarketService durch einen Lock (threading.Lock) serialisieren. Langfristig: Migration zu PostgreSQL für ACID-konforme Parallelzugriffe.</t>
+          <t>WAL-Modus für SQLite aktiviert. threading.Lock im MarketService implementiert. Keine Race-Condition-Fehler während des gesamten Projektzeitraums aufgetreten.</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -822,9 +860,9 @@
           <t>Anwendung neu starten (löst Lock-Situation). Inkonsistente Transaktionen in der DB manuell identifizieren und korrigieren. Bei Wiederholung: SQLite durch PostgreSQL ersetzen.</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>Geschlossen</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -834,7 +872,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>27.06.2026</t>
         </is>
       </c>
     </row>
@@ -884,7 +922,7 @@
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>Wissenstransfer durch regelmäßige Pair-Programming-Sessions und Code-Reviews. Kritische Komponenten (z. B. CoinSyncService) dokumentieren. Aufgaben nicht dauerhaft einer einzigen Person zuordnen.</t>
+          <t>Team hat beide Semester ohne längeren Ausfall durchgehalten. Projekt ist abgeschlossen.</t>
         </is>
       </c>
       <c r="H8" s="12" t="inlineStr">
@@ -897,9 +935,9 @@
           <t>Aufgaben des ausgefallenen Mitglieds im Team neu verteilen. Sprint-Scope reduzieren und Dozenten frühzeitig informieren.</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="J8" s="17" t="inlineStr">
+        <is>
+          <t>Geschlossen</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
@@ -909,7 +947,7 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>27.06.2026</t>
         </is>
       </c>
     </row>
@@ -941,7 +979,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Strikte Definition-of-Done pro Sprint einhalten. Neue Features zunächst ins Backlog aufnehmen und erst in folgenden Sprints planen. Sprint-Ziel zu Beginn schriftlich fixieren.</t>
+          <t>Scope wurde durch konsequente Definition-of-Done kontrolliert. Projekt ist abgeschlossen, kein weiteres Feature-Wachstum möglich.</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
@@ -954,9 +992,9 @@
           <t>Sprint-Scope einfrieren; angefangene, aber nicht fertige Features in separaten Feature-Branches parken und erst nach Abschluss des Kern-Sprints mergen.</t>
         </is>
       </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>Geschlossen</t>
         </is>
       </c>
       <c r="K9" s="11" t="inlineStr">
@@ -966,7 +1004,7 @@
       </c>
       <c r="L9" s="11" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>27.06.2026</t>
         </is>
       </c>
     </row>
@@ -988,17 +1026,17 @@
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>pytest-Framework einrichten und erste Unit-Tests für Services schreiben. CI-Pipeline (z. B. GitHub Actions) einrichten, die Tests bei jedem Push ausführt. Priorität: Tests für Portfolio-Berechnung und Trade-Ausführung.</t>
+          <t>pytest-Framework eingerichtet, 35 Unit- und Integrationstests implementiert (test_market_service.py, test_place_order.py, test_trade_flow.py). CI/CD-Pipeline in GitHub Actions führt Tests bei jedem Push aus. Coverage auf services/market_service.py: 92 % (Ziel ≥80 % erfüllt).</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
@@ -1011,9 +1049,9 @@
           <t>Kritische Pfade (Portfolio, Trade) manuell vor jedem Release durchklicken. Defekte Features sofort im Backlog priorisieren.</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="J10" s="17" t="inlineStr">
+        <is>
+          <t>Geschlossen</t>
         </is>
       </c>
       <c r="K10" s="11" t="inlineStr">
@@ -1023,7 +1061,7 @@
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>27.06.2026</t>
         </is>
       </c>
     </row>
@@ -1068,9 +1106,9 @@
           <t>Scope für betroffenen Sprint reduzieren, vorhandene Ergebnisse dokumentieren und abgeben (lieber vollständige Dokumentation als halbfertiger Code).</t>
         </is>
       </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>Geschlossen</t>
         </is>
       </c>
       <c r="K11" s="11" t="inlineStr">
@@ -1080,7 +1118,7 @@
       </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>27.06.2026</t>
         </is>
       </c>
     </row>

</xml_diff>